<commit_message>
Net concessions into summary in-place rent
Add RollConfig.net_concession (default True): the summary tabs' in-place /
contract rent now uses contract + concession (aggregate.in_place_rent), so a
non-revenue unit nets to 0 and real concessions reduce in-place rent. Affects
Unit Mix Cont Rent + averages, Recent Leases in-place + window averages,
In-Place Rent Annualized, and totals. The Pres. Rent Roll still shows gross
contract and concession in separate columns.

Heritage fixture sets net_concession=False to stay frozen (ALL VALUES MATCH).
Station J Town: 2 BD / 1 BA Cont Rent 207,560 -> 206,425 (model nets out).
Docs + iteration log + saved output updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QgY3cyE49yD2oQoBHHNQL4
</commit_message>
<xml_diff>
--- a/examples/outputs/Rent_Roll_Exhibits_Station_J_Town_07.01.26.xlsx
+++ b/examples/outputs/Rent_Roll_Exhibits_Station_J_Town_07.01.26.xlsx
@@ -954,13 +954,13 @@
         <v>1.154048582995951</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>207560</v>
+        <v>206425</v>
       </c>
       <c r="N7" s="11" t="n">
-        <v>1058.979591836735</v>
+        <v>1053.188775510204</v>
       </c>
       <c r="O7" s="12" t="n">
-        <v>1.114715359828142</v>
+        <v>1.108619763694952</v>
       </c>
       <c r="P7" s="11" t="n">
         <v>1200</v>
@@ -1155,13 +1155,13 @@
         <v>1.178997534921939</v>
       </c>
       <c r="M11" s="17" t="n">
-        <v>386494</v>
+        <v>385359</v>
       </c>
       <c r="N11" s="17" t="n">
-        <v>1067.662983425414</v>
+        <v>1064.527624309392</v>
       </c>
       <c r="O11" s="18" t="n">
-        <v>1.120272463768116</v>
+        <v>1.116982608695652</v>
       </c>
       <c r="P11" s="17" t="n">
         <v>1212.658854166667</v>
@@ -1274,7 +1274,7 @@
       <c r="E21" s="20" t="n"/>
       <c r="F21" s="20" t="n"/>
       <c r="G21" s="24" t="n">
-        <v>4637928</v>
+        <v>4624308</v>
       </c>
     </row>
     <row r="22">
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="W49" s="27" t="n">
-        <v>386494</v>
+        <v>385359</v>
       </c>
     </row>
     <row r="50">
@@ -2106,7 +2106,7 @@
         </is>
       </c>
       <c r="AB66" s="27" t="n">
-        <v>386494</v>
+        <v>385359</v>
       </c>
     </row>
   </sheetData>
@@ -2330,13 +2330,13 @@
         <v>1.159949874686717</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>252609</v>
+        <v>251474</v>
       </c>
       <c r="N7" s="11" t="n">
-        <v>1061.382352941177</v>
+        <v>1056.613445378151</v>
       </c>
       <c r="O7" s="12" t="n">
-        <v>1.117244582043344</v>
+        <v>1.112224679345422</v>
       </c>
       <c r="P7" s="11" t="n">
         <v>1230</v>
@@ -2427,13 +2427,13 @@
         <v>1.178997534921939</v>
       </c>
       <c r="M9" s="17" t="n">
-        <v>386494</v>
+        <v>385359</v>
       </c>
       <c r="N9" s="17" t="n">
-        <v>1067.662983425414</v>
+        <v>1064.527624309392</v>
       </c>
       <c r="O9" s="18" t="n">
-        <v>1.120272463768116</v>
+        <v>1.116982608695652</v>
       </c>
       <c r="P9" s="17" t="inlineStr">
         <is>
@@ -2548,7 +2548,7 @@
       <c r="E19" s="20" t="n"/>
       <c r="F19" s="20" t="n"/>
       <c r="G19" s="24" t="n">
-        <v>4637928</v>
+        <v>4624308</v>
       </c>
     </row>
     <row r="20">
@@ -29286,7 +29286,7 @@
         <v>430452</v>
       </c>
       <c r="V392" s="64" t="n">
-        <v>386494</v>
+        <v>385359</v>
       </c>
       <c r="W392" s="64" t="n">
         <v>-1135</v>

</xml_diff>

<commit_message>
Fix vacant-market comps to be renovation-aware
The vacant market-rent derivation grouped comps by merged floor plan, so a
classic vacant unit could inherit a renovated unit's in-place rent (and vice
versa). Bucket comps by (floor_plan, renovated) instead.

Verified against source: all 21 Station J Town vacants now match the
per-unit-type rule, e.g. stjt2B1 (classic) 1120 -> 965, stjt2B2R (reno) -> 1190.
Heritage regression still passes. Docs + iteration log + saved output updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QgY3cyE49yD2oQoBHHNQL4
</commit_message>
<xml_diff>
--- a/examples/outputs/Rent_Roll_Exhibits_Station_J_Town_07.01.26.xlsx
+++ b/examples/outputs/Rent_Roll_Exhibits_Station_J_Town_07.01.26.xlsx
@@ -945,13 +945,13 @@
         <v>950</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>228040</v>
+        <v>226955</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>1096.346153846154</v>
+        <v>1091.129807692308</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>1.154048582995951</v>
+        <v>1.148557692307692</v>
       </c>
       <c r="M7" s="11" t="n">
         <v>206425</v>
@@ -996,13 +996,13 @@
         <v>950</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>49652</v>
+        <v>49767</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>1128.454545454545</v>
+        <v>1131.068181818182</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>1.187846889952153</v>
+        <v>1.190598086124402</v>
       </c>
       <c r="M8" s="11" t="n">
         <v>45049</v>
@@ -1146,13 +1146,13 @@
         <v>950.78125</v>
       </c>
       <c r="J11" s="17" t="n">
-        <v>430452</v>
+        <v>429482</v>
       </c>
       <c r="K11" s="17" t="n">
-        <v>1120.96875</v>
+        <v>1118.442708333333</v>
       </c>
       <c r="L11" s="18" t="n">
-        <v>1.178997534921939</v>
+        <v>1.176340728567516</v>
       </c>
       <c r="M11" s="17" t="n">
         <v>385359</v>
@@ -1261,7 +1261,7 @@
       <c r="E20" s="20" t="n"/>
       <c r="F20" s="20" t="n"/>
       <c r="G20" s="24" t="n">
-        <v>5165424</v>
+        <v>5153784</v>
       </c>
     </row>
     <row r="21">
@@ -1364,7 +1364,7 @@
         </is>
       </c>
       <c r="W48" s="27" t="n">
-        <v>430452</v>
+        <v>429482</v>
       </c>
     </row>
     <row r="49">
@@ -1705,7 +1705,7 @@
         <v>950</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>1096.346153846154</v>
+        <v>1091.129807692308</v>
       </c>
       <c r="K8" s="38" t="n">
         <v>1094.821428571429</v>
@@ -1771,7 +1771,7 @@
         <v>950</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>1128.454545454545</v>
+        <v>1131.068181818182</v>
       </c>
       <c r="K9" s="38" t="n">
         <v>1131</v>
@@ -1970,7 +1970,7 @@
         <v>950.78125</v>
       </c>
       <c r="J12" s="17" t="n">
-        <v>1120.96875</v>
+        <v>1118.442708333333</v>
       </c>
       <c r="K12" s="42" t="n">
         <v>1124.10773480663</v>
@@ -2096,7 +2096,7 @@
         </is>
       </c>
       <c r="AB65" s="27" t="n">
-        <v>430452</v>
+        <v>429482</v>
       </c>
     </row>
     <row r="66">
@@ -2321,13 +2321,13 @@
         <v>950</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>277692</v>
+        <v>276722</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>1101.952380952381</v>
+        <v>1098.103174603175</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>1.159949874686717</v>
+        <v>1.155898078529658</v>
       </c>
       <c r="M7" s="11" t="n">
         <v>251474</v>
@@ -2418,13 +2418,13 @@
         <v>950.78125</v>
       </c>
       <c r="J9" s="17" t="n">
-        <v>430452</v>
+        <v>429482</v>
       </c>
       <c r="K9" s="17" t="n">
-        <v>1120.96875</v>
+        <v>1118.442708333333</v>
       </c>
       <c r="L9" s="18" t="n">
-        <v>1.178997534921939</v>
+        <v>1.176340728567516</v>
       </c>
       <c r="M9" s="17" t="n">
         <v>385359</v>
@@ -2535,7 +2535,7 @@
       <c r="E18" s="20" t="n"/>
       <c r="F18" s="20" t="n"/>
       <c r="G18" s="24" t="n">
-        <v>5165424</v>
+        <v>5153784</v>
       </c>
     </row>
     <row r="19">
@@ -6474,7 +6474,7 @@
         </is>
       </c>
       <c r="U58" s="58" t="n">
-        <v>1120</v>
+        <v>965</v>
       </c>
       <c r="V58" s="58" t="n">
         <v>0</v>
@@ -11343,7 +11343,7 @@
         </is>
       </c>
       <c r="U129" s="58" t="n">
-        <v>1120</v>
+        <v>965</v>
       </c>
       <c r="V129" s="58" t="n">
         <v>0</v>
@@ -17883,7 +17883,7 @@
         </is>
       </c>
       <c r="U226" s="58" t="n">
-        <v>1075</v>
+        <v>1190</v>
       </c>
       <c r="V226" s="58" t="n">
         <v>0</v>
@@ -19964,7 +19964,7 @@
         </is>
       </c>
       <c r="U256" s="58" t="n">
-        <v>1120</v>
+        <v>965</v>
       </c>
       <c r="V256" s="58" t="n">
         <v>0</v>
@@ -20841,7 +20841,7 @@
         </is>
       </c>
       <c r="U269" s="58" t="n">
-        <v>1120</v>
+        <v>965</v>
       </c>
       <c r="V269" s="58" t="n">
         <v>0</v>
@@ -21927,7 +21927,7 @@
         </is>
       </c>
       <c r="U284" s="58" t="n">
-        <v>1120</v>
+        <v>965</v>
       </c>
       <c r="V284" s="58" t="n">
         <v>0</v>
@@ -25286,7 +25286,7 @@
         </is>
       </c>
       <c r="U333" s="58" t="n">
-        <v>1120</v>
+        <v>965</v>
       </c>
       <c r="V333" s="58" t="n">
         <v>0</v>
@@ -28214,7 +28214,7 @@
         </is>
       </c>
       <c r="U376" s="58" t="n">
-        <v>1120</v>
+        <v>965</v>
       </c>
       <c r="V376" s="58" t="n">
         <v>0</v>
@@ -29283,7 +29283,7 @@
       <c r="S392" s="61" t="n"/>
       <c r="T392" s="61" t="n"/>
       <c r="U392" s="64" t="n">
-        <v>430452</v>
+        <v>429482</v>
       </c>
       <c r="V392" s="64" t="n">
         <v>385359</v>
@@ -34430,7 +34430,7 @@
         </is>
       </c>
       <c r="L82" s="81" t="n">
-        <v>1120</v>
+        <v>965</v>
       </c>
       <c r="M82" s="81">
         <f>Y82</f>
@@ -40003,7 +40003,7 @@
         </is>
       </c>
       <c r="L153" s="81" t="n">
-        <v>1120</v>
+        <v>965</v>
       </c>
       <c r="M153" s="81">
         <f>Y153</f>
@@ -47624,7 +47624,7 @@
         </is>
       </c>
       <c r="L250" s="81" t="n">
-        <v>1075</v>
+        <v>1190</v>
       </c>
       <c r="M250" s="81">
         <f>Y250</f>
@@ -49985,7 +49985,7 @@
         </is>
       </c>
       <c r="L280" s="81" t="n">
-        <v>1120</v>
+        <v>965</v>
       </c>
       <c r="M280" s="81">
         <f>Y280</f>
@@ -50994,7 +50994,7 @@
         </is>
       </c>
       <c r="L293" s="81" t="n">
-        <v>1120</v>
+        <v>965</v>
       </c>
       <c r="M293" s="81">
         <f>Y293</f>
@@ -52170,7 +52170,7 @@
         </is>
       </c>
       <c r="L308" s="81" t="n">
-        <v>1120</v>
+        <v>965</v>
       </c>
       <c r="M308" s="81">
         <f>Y308</f>
@@ -56005,7 +56005,7 @@
         </is>
       </c>
       <c r="L357" s="81" t="n">
-        <v>1120</v>
+        <v>965</v>
       </c>
       <c r="M357" s="81">
         <f>Y357</f>
@@ -59375,7 +59375,7 @@
         </is>
       </c>
       <c r="L400" s="81" t="n">
-        <v>1120</v>
+        <v>965</v>
       </c>
       <c r="M400" s="81">
         <f>Y400</f>

</xml_diff>

<commit_message>
Add occupied $0-rent placeholder rule
An occupied unit carrying $0 contract rent now uses its market rent as a
placeholder in-place rent (no concession). RollConfig.zero_rent_placeholder
(default True). Runs after the vacant-market calc so the $0 unit is never used
as a vacant comp; vacant and non-revenue units are untouched.

Station J Town: L30 (occupied, stjt2A1) contract 0 -> 990 (= market); all 21
vacants still verify against the strict unit-type rule. Heritage frozen (False).
Docs + iteration log + saved output updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QgY3cyE49yD2oQoBHHNQL4
</commit_message>
<xml_diff>
--- a/examples/outputs/Rent_Roll_Exhibits_Station_J_Town_07.01.26.xlsx
+++ b/examples/outputs/Rent_Roll_Exhibits_Station_J_Town_07.01.26.xlsx
@@ -903,13 +903,13 @@
         <v>1.179983660130719</v>
       </c>
       <c r="M6" s="11" t="n">
-        <v>59493</v>
+        <v>60483</v>
       </c>
       <c r="N6" s="11" t="n">
-        <v>929.578125</v>
+        <v>945.046875</v>
       </c>
       <c r="O6" s="12" t="n">
-        <v>1.093621323529412</v>
+        <v>1.111819852941176</v>
       </c>
       <c r="P6" s="11" t="n">
         <v>1050</v>
@@ -1155,13 +1155,13 @@
         <v>1.176340728567516</v>
       </c>
       <c r="M11" s="17" t="n">
-        <v>385359</v>
+        <v>386349</v>
       </c>
       <c r="N11" s="17" t="n">
-        <v>1064.527624309392</v>
+        <v>1067.262430939227</v>
       </c>
       <c r="O11" s="18" t="n">
-        <v>1.116982608695652</v>
+        <v>1.119852173913043</v>
       </c>
       <c r="P11" s="17" t="n">
         <v>1212.658854166667</v>
@@ -1274,7 +1274,7 @@
       <c r="E21" s="20" t="n"/>
       <c r="F21" s="20" t="n"/>
       <c r="G21" s="24" t="n">
-        <v>4624308</v>
+        <v>4636188</v>
       </c>
     </row>
     <row r="22">
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="W49" s="27" t="n">
-        <v>385359</v>
+        <v>386349</v>
       </c>
     </row>
     <row r="50">
@@ -1645,37 +1645,37 @@
         <v>1004.609375</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>929.578125</v>
+        <v>945.046875</v>
       </c>
       <c r="M7" s="39" t="n">
-        <v>0.9253130103429504</v>
+        <v>0.9407107862197682</v>
       </c>
       <c r="N7" s="38" t="n">
-        <v>882</v>
+        <v>981</v>
       </c>
       <c r="O7" s="40" t="n">
         <v>10</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>863.75</v>
+        <v>987.5</v>
       </c>
       <c r="Q7" s="40" t="n">
         <v>8</v>
       </c>
       <c r="R7" s="11" t="n">
-        <v>823.3333333333334</v>
+        <v>988.3333333333334</v>
       </c>
       <c r="S7" s="40" t="n">
         <v>6</v>
       </c>
       <c r="T7" s="11" t="n">
-        <v>655</v>
+        <v>985</v>
       </c>
       <c r="U7" s="40" t="n">
         <v>3</v>
       </c>
       <c r="V7" s="11" t="n">
-        <v>655</v>
+        <v>985</v>
       </c>
       <c r="W7" s="40" t="n">
         <v>3</v>
@@ -1976,10 +1976,10 @@
         <v>1124.10773480663</v>
       </c>
       <c r="L12" s="17" t="n">
-        <v>1064.527624309392</v>
+        <v>1067.262430939227</v>
       </c>
       <c r="M12" s="43" t="n">
-        <v>0.9469978644818358</v>
+        <v>0.9494307332764844</v>
       </c>
       <c r="N12" s="42" t="inlineStr">
         <is>
@@ -2106,7 +2106,7 @@
         </is>
       </c>
       <c r="AB66" s="27" t="n">
-        <v>385359</v>
+        <v>386349</v>
       </c>
     </row>
   </sheetData>
@@ -2281,13 +2281,13 @@
         <v>1.179983660130719</v>
       </c>
       <c r="M6" s="11" t="n">
-        <v>59493</v>
+        <v>60483</v>
       </c>
       <c r="N6" s="11" t="n">
-        <v>929.578125</v>
+        <v>945.046875</v>
       </c>
       <c r="O6" s="12" t="n">
-        <v>1.093621323529412</v>
+        <v>1.111819852941176</v>
       </c>
       <c r="P6" s="11" t="n">
         <v>1050</v>
@@ -2427,13 +2427,13 @@
         <v>1.176340728567516</v>
       </c>
       <c r="M9" s="17" t="n">
-        <v>385359</v>
+        <v>386349</v>
       </c>
       <c r="N9" s="17" t="n">
-        <v>1064.527624309392</v>
+        <v>1067.262430939227</v>
       </c>
       <c r="O9" s="18" t="n">
-        <v>1.116982608695652</v>
+        <v>1.119852173913043</v>
       </c>
       <c r="P9" s="17" t="inlineStr">
         <is>
@@ -2548,7 +2548,7 @@
       <c r="E19" s="20" t="n"/>
       <c r="F19" s="20" t="n"/>
       <c r="G19" s="24" t="n">
-        <v>4624308</v>
+        <v>4636188</v>
       </c>
     </row>
     <row r="20">
@@ -28824,7 +28824,7 @@
         <v>990</v>
       </c>
       <c r="V385" s="58" t="n">
-        <v>0</v>
+        <v>990</v>
       </c>
       <c r="W385" s="58" t="n">
         <v>0</v>
@@ -29286,7 +29286,7 @@
         <v>429482</v>
       </c>
       <c r="V392" s="64" t="n">
-        <v>385359</v>
+        <v>386349</v>
       </c>
       <c r="W392" s="64" t="n">
         <v>-1135</v>
@@ -60096,7 +60096,7 @@
         <v/>
       </c>
       <c r="Y409" s="81" t="n">
-        <v>0</v>
+        <v>990</v>
       </c>
     </row>
     <row r="410">

</xml_diff>